<commit_message>
Distinguish between pay period and calendar month.
</commit_message>
<xml_diff>
--- a/tests/output/basic.xlsx
+++ b/tests/output/basic.xlsx
@@ -14,50 +14,55 @@
     <ns0:row r="1">
       <ns0:c r="A1" t="inlineStr">
         <ns0:is>
-          <ns0:t>yyyy-mm</ns0:t>
+          <ns0:t>payroll period</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="B1" t="inlineStr">
         <ns0:is>
-          <ns0:t>gross salary</ns0:t>
+          <ns0:t>calendar month</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C1" t="inlineStr">
         <ns0:is>
-          <ns0:t>tax deducted</ns0:t>
+          <ns0:t>gross salary</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D1" t="inlineStr">
         <ns0:is>
-          <ns0:t>ni deducted</ns0:t>
+          <ns0:t>tax deducted</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E1" t="inlineStr">
         <ns0:is>
-          <ns0:t>pension deducted</ns0:t>
+          <ns0:t>ni deducted</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F1" t="inlineStr">
         <ns0:is>
-          <ns0:t>net salary</ns0:t>
+          <ns0:t>pension deducted</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G1" t="inlineStr">
         <ns0:is>
-          <ns0:t>employers pension</ns0:t>
+          <ns0:t>net salary</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H1" t="inlineStr">
         <ns0:is>
-          <ns0:t>deductions total</ns0:t>
+          <ns0:t>employers pension</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I1" t="inlineStr">
         <ns0:is>
+          <ns0:t>deductions total</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J1" t="inlineStr">
+        <ns0:is>
           <ns0:t>gross minus deductions and net</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J1" t="inlineStr">
+      <ns0:c r="K1" t="inlineStr">
         <ns0:is>
           <ns0:t>valid</ns0:t>
         </ns0:is>
@@ -69,32 +74,37 @@
           <ns0:t>2026-03</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B2">
+      <ns0:c r="B2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2026-06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2">
         <ns0:v>1234.56</ns0:v>
       </ns0:c>
-      <ns0:c r="C2">
+      <ns0:c r="D2">
         <ns0:v>234.00</ns0:v>
       </ns0:c>
-      <ns0:c r="D2">
+      <ns0:c r="E2">
         <ns0:v>0.56</ns0:v>
       </ns0:c>
-      <ns0:c r="E2">
+      <ns0:c r="F2">
         <ns0:v>100.00</ns0:v>
       </ns0:c>
-      <ns0:c r="F2">
+      <ns0:c r="G2">
         <ns0:v>900.00</ns0:v>
       </ns0:c>
-      <ns0:c r="G2">
+      <ns0:c r="H2">
         <ns0:v>200.00</ns0:v>
       </ns0:c>
-      <ns0:c r="H2">
-        <ns0:f>SUM(C2:E2)</ns0:f>
-      </ns0:c>
       <ns0:c r="I2">
-        <ns0:f>B2-H2-F2</ns0:f>
+        <ns0:f>SUM(D2:F2)</ns0:f>
       </ns0:c>
       <ns0:c r="J2">
-        <ns0:f>ABS(I2)&lt;0.01</ns0:f>
+        <ns0:f>C2-I2-G2</ns0:f>
+      </ns0:c>
+      <ns0:c r="K2">
+        <ns0:f>ABS(J2)&lt;0.01</ns0:f>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>

</xml_diff>